<commit_message>
feat: added exceljs for excel file generation and started the genreports functionality
</commit_message>
<xml_diff>
--- a/backend/templates/Supply and Market Profile Report Template.xlsx
+++ b/backend/templates/Supply and Market Profile Report Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeric\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeric\Desktop\AgriTrack\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F09DD676-855D-42E8-A4C1-FC29F107358E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BB37ED-4D39-4593-AAD1-AAA7A1B26FB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Department of Agriculture</t>
   </si>
@@ -113,24 +113,12 @@
   <si>
     <t>To date</t>
   </si>
-  <si>
-    <t>Prepared by:</t>
-  </si>
-  <si>
-    <t>Noted by:</t>
-  </si>
-  <si>
-    <t>RUBY V. ARENAS</t>
-  </si>
-  <si>
-    <t>City Agriculturist</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -215,19 +203,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -329,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -394,52 +369,31 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -789,12 +743,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -814,12 +768,12 @@
       <c r="U1" s="1"/>
     </row>
     <row r="2" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -839,12 +793,12 @@
       <c r="U2" s="1"/>
     </row>
     <row r="3" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -890,10 +844,10 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="28"/>
+      <c r="C5" s="25"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -917,10 +871,10 @@
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="28"/>
+      <c r="C6" s="25"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -944,8 +898,8 @@
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="28"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="25"/>
       <c r="D7" s="5"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -989,94 +943,94 @@
       <c r="U8" s="6"/>
     </row>
     <row r="9" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="36" t="s">
+      <c r="E9" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="36" t="s">
+      <c r="F9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="36" t="s">
+      <c r="G9" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="36" t="s">
+      <c r="H9" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="36" t="s">
+      <c r="I9" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="36" t="s">
+      <c r="J9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="36" t="s">
+      <c r="K9" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="38" t="s">
+      <c r="L9" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="32"/>
-      <c r="N9" s="36" t="s">
+      <c r="M9" s="28"/>
+      <c r="N9" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="36" t="s">
+      <c r="O9" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="P9" s="37" t="s">
+      <c r="P9" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="Q9" s="36" t="s">
+      <c r="Q9" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="R9" s="36" t="s">
+      <c r="R9" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="S9" s="36" t="s">
+      <c r="S9" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="T9" s="36" t="s">
+      <c r="T9" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="U9" s="36" t="s">
+      <c r="U9" s="23" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="25" t="s">
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="22" t="s">
         <v>27</v>
       </c>
       <c r="M10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="N10" s="26"/>
-      <c r="O10" s="26"/>
-      <c r="P10" s="26"/>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="26"/>
-      <c r="S10" s="26"/>
-      <c r="T10" s="26"/>
-      <c r="U10" s="26"/>
+      <c r="N10" s="24"/>
+      <c r="O10" s="24"/>
+      <c r="P10" s="24"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="24"/>
+      <c r="T10" s="24"/>
+      <c r="U10" s="24"/>
     </row>
     <row r="11" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
@@ -1104,120 +1058,36 @@
     <row r="12" spans="1:21" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:21" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="R14" s="1"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
+      <c r="A14" s="2"/>
     </row>
     <row r="15" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="1"/>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
     </row>
     <row r="16" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="24"/>
-      <c r="Q16" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="R16" s="28"/>
-      <c r="S16" s="28"/>
-      <c r="T16" s="21"/>
-    </row>
-    <row r="17" spans="1:20" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
-      <c r="P17" s="24"/>
-      <c r="Q17" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="R17" s="28"/>
-      <c r="S17" s="28"/>
-      <c r="T17" s="1"/>
-    </row>
-    <row r="18" spans="1:20" ht="13.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="21"/>
+    </row>
+    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+    </row>
+    <row r="18" spans="1:3" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:20" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="21" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="24" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="31" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:3" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="33" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="34" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="35" ht="13.8" x14ac:dyDescent="0.3"/>
@@ -1349,7 +1219,7 @@
     <row r="104" spans="1:21" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="105" spans="1:21" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="106" spans="1:21" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="107" spans="1:21" ht="15.6" x14ac:dyDescent="0.3"/>
+    <row r="107" spans="1:21" ht="13.8" x14ac:dyDescent="0.3"/>
     <row r="108" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
@@ -7763,14 +7633,13 @@
       <c r="U386" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="26">
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="J9:J10"/>
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="A9:A10"/>
@@ -7781,10 +7650,6 @@
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="T9:T10"/>
     <mergeCell ref="U9:U10"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="Q17:S17"/>
     <mergeCell ref="N9:N10"/>
     <mergeCell ref="O9:O10"/>
     <mergeCell ref="P9:P10"/>
@@ -7794,6 +7659,7 @@
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: improve Excel report generation by sorting records alphabetically and enhancing data insertion logic
</commit_message>
<xml_diff>
--- a/backend/templates/Supply and Market Profile Report Template.xlsx
+++ b/backend/templates/Supply and Market Profile Report Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeric\Desktop\AgriTrack\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BB37ED-4D39-4593-AAD1-AAA7A1B26FB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F11DD4-BD03-4BE0-BA04-3A7D174D7A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -304,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -372,21 +372,10 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -396,6 +385,18 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -743,12 +744,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -768,12 +769,12 @@
       <c r="U1" s="1"/>
     </row>
     <row r="2" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -793,12 +794,12 @@
       <c r="U2" s="1"/>
     </row>
     <row r="3" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -844,10 +845,10 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="25"/>
+      <c r="C5" s="24"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -871,10 +872,10 @@
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="25"/>
+      <c r="C6" s="24"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -898,8 +899,8 @@
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="29"/>
-      <c r="C7" s="25"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="33"/>
       <c r="D7" s="5"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -943,94 +944,94 @@
       <c r="U8" s="6"/>
     </row>
     <row r="9" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="23" t="s">
+      <c r="J9" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="23" t="s">
+      <c r="K9" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="27" t="s">
+      <c r="L9" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="28"/>
-      <c r="N9" s="23" t="s">
+      <c r="M9" s="31"/>
+      <c r="N9" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="23" t="s">
+      <c r="O9" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="P9" s="26" t="s">
+      <c r="P9" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="Q9" s="23" t="s">
+      <c r="Q9" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="R9" s="23" t="s">
+      <c r="R9" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="S9" s="23" t="s">
+      <c r="S9" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="T9" s="23" t="s">
+      <c r="T9" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="U9" s="23" t="s">
+      <c r="U9" s="28" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
+      <c r="A10" s="29"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
       <c r="L10" s="22" t="s">
         <v>27</v>
       </c>
       <c r="M10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="N10" s="24"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="24"/>
-      <c r="R10" s="24"/>
-      <c r="S10" s="24"/>
-      <c r="T10" s="24"/>
-      <c r="U10" s="24"/>
+      <c r="N10" s="29"/>
+      <c r="O10" s="29"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="29"/>
+      <c r="R10" s="29"/>
+      <c r="S10" s="29"/>
+      <c r="T10" s="29"/>
+      <c r="U10" s="29"/>
     </row>
     <row r="11" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
@@ -1066,7 +1067,7 @@
     <row r="16" spans="1:21" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A16" s="21"/>
     </row>
-    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
     </row>
     <row r="18" spans="1:3" ht="13.8" x14ac:dyDescent="0.3">
@@ -7633,13 +7634,15 @@
       <c r="U386" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
+  <mergeCells count="25">
+    <mergeCell ref="T9:T10"/>
+    <mergeCell ref="U9:U10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="P9:P10"/>
+    <mergeCell ref="Q9:Q10"/>
+    <mergeCell ref="R9:R10"/>
+    <mergeCell ref="S9:S10"/>
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="A9:A10"/>
@@ -7648,18 +7651,15 @@
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="F9:F10"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="P9:P10"/>
-    <mergeCell ref="Q9:Q10"/>
-    <mergeCell ref="R9:R10"/>
-    <mergeCell ref="S9:S10"/>
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="I9:I10"/>
     <mergeCell ref="J9:J10"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>